<commit_message>
docs: PRD, content pipeline script, and compliance requirements
- PRD.md updated with v0.2–v1.0 roadmap and privacy/legal framework
- scripts/csv_to_json.py content pipeline for Excel→JSON conversion
- Content/clio_content.xlsx source workbook
- docs/requirements/REQ-001-content-safety-audit.md
- docs/requirements/REQ-002-appstore-compliance.md
</commit_message>
<xml_diff>
--- a/Content/clio_content.xlsx
+++ b/Content/clio_content.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="nudges" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="signals" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="insights" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +61,11 @@
         <fgColor rgb="002E9E6B"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E57C4A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -73,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -85,6 +91,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -559,10 +568,6 @@
       <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -598,10 +603,6 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -637,10 +638,6 @@
       <c r="G4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -681,9 +678,6 @@
           <t>cramps</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -719,10 +713,6 @@
       <c r="G6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -763,9 +753,6 @@
           <t>cramps</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -806,9 +793,6 @@
           <t>bloating</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -849,9 +833,6 @@
           <t>fatigue</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -887,10 +868,6 @@
       <c r="G10" t="n">
         <v>0</v>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -926,10 +903,6 @@
       <c r="G11" t="n">
         <v>0</v>
       </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -965,10 +938,6 @@
       <c r="G12" t="n">
         <v>0</v>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1004,10 +973,6 @@
       <c r="G13" t="n">
         <v>0</v>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1048,9 +1013,6 @@
           <t>acne</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1086,10 +1048,6 @@
       <c r="G15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1125,10 +1083,6 @@
       <c r="G16" t="n">
         <v>0</v>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1164,10 +1118,6 @@
       <c r="G17" t="n">
         <v>0</v>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1203,10 +1153,6 @@
       <c r="G18" t="n">
         <v>0</v>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1247,9 +1193,6 @@
           <t>mittelschmerz</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1290,9 +1233,6 @@
           <t>dischargeChanges</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1328,10 +1268,6 @@
       <c r="G21" t="n">
         <v>0</v>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1367,10 +1303,6 @@
       <c r="G22" t="n">
         <v>0</v>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1406,9 +1338,6 @@
       <c r="G23" t="n">
         <v>0</v>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1449,9 +1378,6 @@
           <t>insomnia</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1492,9 +1418,6 @@
           <t>bloating</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1535,9 +1458,6 @@
           <t>brainFog</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1578,9 +1498,6 @@
           <t>foodCravings</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1621,9 +1538,6 @@
           <t>anxious,irritable,sad</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1664,9 +1578,6 @@
           <t>breastTenderness</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1813,15 +1724,9 @@
       <c r="H2" t="n">
         <v>21</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="b">
         <v>1</v>
       </c>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1857,18 +1762,12 @@
       <c r="G3" t="n">
         <v>3</v>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
         <v>35</v>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="b">
         <v>1</v>
       </c>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1904,18 +1803,12 @@
       <c r="G4" t="n">
         <v>3</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
         <v>7</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="b">
         <v>1</v>
       </c>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1951,18 +1844,12 @@
       <c r="G5" t="n">
         <v>3</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
         <v>7</v>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="b">
         <v>1</v>
       </c>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1998,20 +1885,14 @@
       <c r="G6" t="n">
         <v>2</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>cramps</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="b">
         <v>1</v>
       </c>
-      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2047,20 +1928,14 @@
       <c r="G7" t="n">
         <v>2</v>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>fatigue</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="b">
         <v>1</v>
       </c>
-      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2096,20 +1971,14 @@
       <c r="G8" t="n">
         <v>2</v>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>bloating</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="b">
         <v>1</v>
       </c>
-      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2145,20 +2014,14 @@
       <c r="G9" t="n">
         <v>2</v>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>insomnia</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
       <c r="N9" t="b">
         <v>1</v>
       </c>
-      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2194,20 +2057,14 @@
       <c r="G10" t="n">
         <v>2</v>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>brainFog</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
       <c r="N10" t="b">
         <v>1</v>
       </c>
-      <c r="O10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2315,8 +2172,6 @@
           <t>cramps_escalating</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2352,8 +2207,6 @@
           <t>heavy_flow_majority</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2389,8 +2242,6 @@
           <t>cramps_follicular</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2426,8 +2277,6 @@
           <t>severe_cluster</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2527,7 +2376,6 @@
           <t>https://www.acog.org/womens-health/faqs/abnormal-uterine-bleeding</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>US</t>
@@ -2570,7 +2418,6 @@
           <t>https://www.acog.org/womens-health/faqs/endometriosis</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>US</t>
@@ -2613,7 +2460,6 @@
           <t>https://www.acog.org/womens-health/faqs/polycystic-ovary-syndrome</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>US</t>
@@ -2656,7 +2502,6 @@
           <t>https://iapmd.org</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>global</t>
@@ -2699,7 +2544,6 @@
           <t>https://iapmd.org/crisis-support</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>global</t>
@@ -2742,7 +2586,6 @@
           <t>https://www.endofound.org</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>US</t>
@@ -2832,7 +2675,6 @@
           <t>https://www.verity-pcos.org.uk</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>UK</t>
@@ -2875,7 +2717,6 @@
           <t>https://www.pcosaa.org</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>US</t>
@@ -2918,7 +2759,6 @@
           <t>https://www.nhs.uk/conditions/periods/</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>UK</t>
@@ -2961,7 +2801,6 @@
           <t>https://www.nhs.uk/conditions/endometriosis/</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>UK</t>
@@ -3004,7 +2843,6 @@
           <t>https://www.nhs.uk/conditions/polycystic-ovary-syndrome-pcos/</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>UK</t>
@@ -3047,7 +2885,6 @@
           <t>https://medlineplus.gov/menstruation.html</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>US</t>
@@ -3090,7 +2927,6 @@
           <t>https://medlineplus.gov/endometriosis.html</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>US</t>
@@ -3133,7 +2969,6 @@
           <t>https://medlineplus.gov/premenstrualdysphoricdisorder.html</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>US</t>
@@ -3411,7 +3246,6 @@
           <t>https://www.mind.org.uk</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>UK</t>
@@ -3472,6 +3306,1219 @@
       <c r="I23" t="inlineStr">
         <is>
           <t>mental_health,mood</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>symptom</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>prevalence</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>percentage_string</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>valence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>insight.menstrual.cramps</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>cramps</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>very_common</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>around 70%</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Cramps are one of the most reported period symptoms. Pain that stops you doing normal activities is worth discussing with a doctor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>insight.menstrual.bloating</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>bloating</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>very_common</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>around 65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>insight.menstrual.backPain</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>backPain</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>around 45%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>insight.menstrual.fatigue</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>fatigue</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>very_common</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>around 60%</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Iron loss during menstruation contributes to fatigue for many people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>insight.menstrual.headache</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>around 35%</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Hormone shifts at the start of the cycle can trigger headaches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>insight.menstrual.nausea</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>nausea</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>fairly_common</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>around 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>insight.menstrual.breastTenderness</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>breastTenderness</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>fairly_common</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>around 25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>insight.menstrual.insomnia</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>insomnia</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>fairly_common</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>around 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>insight.menstrual.foodCravings</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>foodCravings</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>around 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>insight.menstrual.brainFog</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>brainFog</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fairly_common</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>around 25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>insight.menstrual.acne</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>acne</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>fairly_common</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>around 30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>insight.follicular.fatigue</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>fatigue</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>follicular</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>less_common</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>around 15%</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Fatigue is less typical in the follicular phase as oestrogen rises. If it is persistent, worth noting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>insight.follicular.headache</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>follicular</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>less_common</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>around 10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>insight.follicular.acne</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>acne</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>follicular</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>fairly_common</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>around 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>insight.follicular.bloating</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>bloating</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>follicular</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>less_common</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>around 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>insight.follicular.cramps</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>cramps</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>follicular</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>around 5-10%</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Cramps outside your period are less typical. If this is consistent it is worth mentioning to a doctor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>insight.follicular.highEnergy</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>highEnergy</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>follicular</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>around 55%</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Many people notice a natural energy lift during the follicular phase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>insight.follicular.brainFog</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>brainFog</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>follicular</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>less_common</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>around 10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>insight.ovulatory.mittelschmerz</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>mittelschmerz</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ovulatory</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>around 40%</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>A brief one-sided ache or twinge around ovulation is very common and harmless.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>insight.ovulatory.dischargeChanges</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>dischargeChanges</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ovulatory</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>very_common</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>around 70%</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Discharge changes around ovulation are a normal hormonal signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>insight.ovulatory.bloating</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>bloating</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ovulatory</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>fairly_common</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>around 25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>insight.ovulatory.headache</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ovulatory</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>fairly_common</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>around 20%</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>The oestrogen peak before ovulation can trigger headaches in some people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>insight.ovulatory.breastTenderness</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>breastTenderness</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ovulatory</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>fairly_common</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>around 30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>insight.ovulatory.highEnergy</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>highEnergy</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ovulatory</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>very_common</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>around 60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>insight.luteal.breastTenderness</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>breastTenderness</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>very_common</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>around 60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>insight.luteal.bloating</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>bloating</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>very_common</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>around 65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>insight.luteal.foodCravings</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>foodCravings</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>very_common</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>around 60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>insight.luteal.fatigue</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>fatigue</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>around 45%</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Energy often dips in the late luteal phase as progesterone peaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>insight.luteal.insomnia</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>insomnia</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>around 35%</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Progesterone fluctuations can affect sleep quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>insight.luteal.brainFog</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>brainFog</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>around 40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>insight.luteal.acne</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>acne</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>around 45%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>insight.luteal.headache</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>headache</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>around 35%</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Pre-menstrual headaches caused by the oestrogen drop before your period are very common.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>insight.luteal.cramps</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>cramps</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>fairly_common</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>around 20%</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Some cramping in the late luteal phase is common as the uterus prepares.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>insight.luteal.appetiteChanges</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>appetiteChanges</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>around 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>insight.luteal.backPain</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>backPain</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>fairly_common</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>around 25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>insight.mood.luteal.negative</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>mood</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>luteal</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>very_common</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>around 75%</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Mood changes in the luteal phase are one of the most reported cycle experiences.</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>insight.mood.menstrual.negative</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>mood</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>menstrual</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>around 50%</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>insight.mood.follicular.positive</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>mood</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>follicular</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>around 55%</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Rising oestrogen in this phase often lifts mood and energy.</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>insight.mood.ovulatory.positive</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>mood</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ovulatory</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>around 55%</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Rising oestrogen in this phase often lifts mood and energy.</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
     </row>

</xml_diff>